<commit_message>
Updated BRA model - 2025-09-08 20:10
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C2C3176-B459-4A0F-8CC2-E3F347B90B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5173816-9D61-49A4-A0A0-02D429BFB3A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9BF348C-8707-4031-88A8-91860342D3A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DE1E966-A624-4204-9E49-977A1F3812FC}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC627863-8385-4420-B742-E646B908FC34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{812A7BAC-F1DB-4E5D-8E29-EB4F0A4905BE}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B80FAF24-F9BC-43F0-AB4C-0F2D0C4EFE77}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC70E0DC-277E-4B5F-9E32-EA330CAEFE3E}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-08 23:31
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E3E41C6-D236-417B-BD35-F45E7649D7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F77FAF38-999F-4EC3-B234-839EA1C940A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90A7A860-0975-4DAC-B683-112C7D32E4B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FB2B0BB-F21C-4AC6-81B1-69DF7CD8293B}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAAC38A3-DCB1-4357-B503-DCC59567B57F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DBE3ACC-12D9-4621-81F8-1E110C1C535D}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C49D24D0-4286-4767-9CB0-3A90B41CD17E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9546808B-329C-4321-B997-C2D730BC23EA}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-09 22:31
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F77FAF38-999F-4EC3-B234-839EA1C940A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C51771C6-82B4-4C1E-AA54-670BC3C9500D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FB2B0BB-F21C-4AC6-81B1-69DF7CD8293B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99FED5AB-ED55-408F-9B14-5809A0CF96AF}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DBE3ACC-12D9-4621-81F8-1E110C1C535D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76083E65-338F-4470-9A5C-6320CF406D66}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9546808B-329C-4321-B997-C2D730BC23EA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B096C26C-18D5-4E5A-BD33-C0DA0FB01294}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-10 08:33
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C51771C6-82B4-4C1E-AA54-670BC3C9500D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{25A5C76F-C574-4169-805E-F5FC52650135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99FED5AB-ED55-408F-9B14-5809A0CF96AF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ABCAE8A-3674-4086-B22C-A5C59A22FA1B}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76083E65-338F-4470-9A5C-6320CF406D66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04D1AF88-6C3F-4DAB-8AE9-6DE975EE0D7A}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B096C26C-18D5-4E5A-BD33-C0DA0FB01294}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0115B320-8727-43F6-8A46-76CCB16E42EA}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-10 23:58
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94A9FA11-5F4C-498D-B3A8-5A4FDC16E5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A81C3B8-C9AE-482C-9EBF-2BF7633F234D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D836F4DA-1E54-4F1A-9278-C6175CB791BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD17C855-5215-4813-BC64-985A3503C4A4}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71D73EE1-9FAD-4809-8A52-06DBC0A9C49F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A724DDF-C219-4F54-8951-DD2DBEE113BC}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{492BC9BE-25C6-4471-8658-E862BEDDA619}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4F8EFD-CAD0-4E92-A03E-22E79D4E3FE1}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-11 00:03
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A81C3B8-C9AE-482C-9EBF-2BF7633F234D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD762BCA-A3FF-42B7-B4E3-A7F2E2C0A2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD17C855-5215-4813-BC64-985A3503C4A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38559C4D-A515-420F-8C21-E5B9BC0FF3A7}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A724DDF-C219-4F54-8951-DD2DBEE113BC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67C9497E-D090-4E17-A5C1-0ECF3072D382}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4F8EFD-CAD0-4E92-A03E-22E79D4E3FE1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FB723D6-A428-46E9-931A-83C98A81C315}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-11 11:58
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD762BCA-A3FF-42B7-B4E3-A7F2E2C0A2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0AE67BC0-CD25-4165-BF6D-DA19C659B6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38559C4D-A515-420F-8C21-E5B9BC0FF3A7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87E4AB3F-0354-4CA0-A2F0-B16936BD99D3}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67C9497E-D090-4E17-A5C1-0ECF3072D382}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA7D12F2-77DB-4134-9068-41B8BD6E1021}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FB723D6-A428-46E9-931A-83C98A81C315}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71769D25-C890-483F-BF08-E26B414475CF}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-11 12:01
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0AE67BC0-CD25-4165-BF6D-DA19C659B6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{322BD2EB-8A9B-4216-9099-63EB88C6E84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87E4AB3F-0354-4CA0-A2F0-B16936BD99D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{999C48E5-5866-4846-8030-B22AB54E8ABA}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA7D12F2-77DB-4134-9068-41B8BD6E1021}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FD02540-5899-4893-8668-98832A1C51D7}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71769D25-C890-483F-BF08-E26B414475CF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D0B21EC-4217-4ACC-B2CB-F844601BF409}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-11 13:15
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{322BD2EB-8A9B-4216-9099-63EB88C6E84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{857DC2C1-8FF4-4E7E-A871-78345AB69018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8768,7 +8768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{999C48E5-5866-4846-8030-B22AB54E8ABA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F51576B2-2D70-4F7E-8D2D-5A89CE566E2D}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FD02540-5899-4893-8668-98832A1C51D7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{314FA4A1-658D-49D7-A2E1-F604BF105430}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D0B21EC-4217-4ACC-B2CB-F844601BF409}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF941244-AC6F-4122-A03C-D49788512BDC}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-11 18:46
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{472CDAC6-83F8-4C94-9ECD-FD9EE46282BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D27B0670-4E1A-4C61-B226-9655B8EC68FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="21600" windowHeight="12682" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc" sheetId="7" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5412" uniqueCount="1261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5414" uniqueCount="1261">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -5450,7 +5450,9 @@
       <c r="F8" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="1"/>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="str">
@@ -5486,7 +5488,9 @@
       <c r="F9" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="K9" s="1"/>
@@ -8768,7 +8772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95AAD808-3052-4A11-A2BD-E5B6CF363F20}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F400B4D-90DA-4BFC-91C8-BF306082E914}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10876,7 +10880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0436BE9-09AC-410D-9639-9C8BDBB523F2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3586EA31-90F7-4296-92E5-87175DBA753E}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28400,7 +28404,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0609CF0E-C7AB-4DA1-A746-BD34C86710C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{415FC8ED-B32F-4853-9085-E8E65DCFE9B8}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-13 16:41
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D27B0670-4E1A-4C61-B226-9655B8EC68FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8E922CB-A3BB-4633-A14F-450D15CA98CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8772,7 +8772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F400B4D-90DA-4BFC-91C8-BF306082E914}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{967BC00D-3172-4551-84AB-DC4819178B34}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10880,7 +10880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3586EA31-90F7-4296-92E5-87175DBA753E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B62AAA80-791D-4EB1-A3E6-8A16E613503D}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28404,7 +28404,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{415FC8ED-B32F-4853-9085-E8E65DCFE9B8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{521912C6-C159-4057-B655-DE82A22AAE9D}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-14 13:14
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8E922CB-A3BB-4633-A14F-450D15CA98CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8FB1FC59-B9C2-46C3-AC75-1D190AD47D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8772,7 +8772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{967BC00D-3172-4551-84AB-DC4819178B34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A44D4F4D-978A-4B7D-AB75-DC63F1FF9B30}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10880,7 +10880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B62AAA80-791D-4EB1-A3E6-8A16E613503D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E111444-1059-457E-8530-0801F73869E3}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28404,7 +28404,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{521912C6-C159-4057-B655-DE82A22AAE9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FF9591D-90D1-4960-992C-7BE6B9769451}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-14 13:40
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8FB1FC59-B9C2-46C3-AC75-1D190AD47D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{207FEB6C-CB47-41C3-8C3A-0BC603BCEDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8772,7 +8772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A44D4F4D-978A-4B7D-AB75-DC63F1FF9B30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FB094AA-F3C7-482C-8EDF-E9366F5A201D}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10880,7 +10880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E111444-1059-457E-8530-0801F73869E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64F8A8A2-79D8-43A4-B15F-AC53F8FAF865}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28404,7 +28404,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FF9591D-90D1-4960-992C-7BE6B9769451}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E476E86D-6072-47C0-8B3D-E8440AAB4B82}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-14 13:49
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{207FEB6C-CB47-41C3-8C3A-0BC603BCEDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B6683C8-A297-43C0-8A3A-5A0A86CFF9A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8772,7 +8772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FB094AA-F3C7-482C-8EDF-E9366F5A201D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9781D36-AD64-42D7-9E26-8FC9634F8B3F}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10880,7 +10880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64F8A8A2-79D8-43A4-B15F-AC53F8FAF865}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5921A6F9-9DBF-4A64-8DF3-F94EC5D731F8}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28404,7 +28404,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E476E86D-6072-47C0-8B3D-E8440AAB4B82}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{727CCDCA-41C4-4E27-83FB-19566382DBC2}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-14 18:31
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_BRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B6683C8-A297-43C0-8A3A-5A0A86CFF9A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B58C54FC-9857-4950-A706-33D46631625B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8772,7 +8772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9781D36-AD64-42D7-9E26-8FC9634F8B3F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{551C3B0E-F800-484C-AD01-458A00903AD7}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10880,7 +10880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5921A6F9-9DBF-4A64-8DF3-F94EC5D731F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F46191A-5DEA-4F41-A931-C3C9E7047610}">
   <dimension ref="B9:AB263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28404,7 +28404,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{727CCDCA-41C4-4E27-83FB-19566382DBC2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6272F942-86D2-4DF4-AF07-2898B00D0ACC}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>